<commit_message>
ДСУП: РЕ / КУП от шины PE — patch_dsup.py (шаг 17), SXDRAW v3.23
Книга: «Справочная» DF коды ДСУП, «Однолинейка» CJ:CK; строка ДСУП без QF и клемм, фаза PE.
SXDRAW: ДСУП на уровне общей шины PE, блок «_КУП», отводы РЕ от КУП (образец ЩР-2, 098).
Шаблон и пример пропатчены. Заодно — несохранённые правки 15.10 (узел КМ, cmd, СОСТОЯНИЕ).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/1_Таблицы_Excel/Каталог_общий.xlsx
+++ b/1_Таблицы_Excel/Каталог_общий.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\02_Справочники_CAD_Revit\odnolineyka\1_Таблицы_Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F90BB689-9568-4C0A-B548-A291FB1AFAE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C49E891-9CBE-40E7-9264-800F2F1AF83A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="296">
   <si>
     <t>Общий каталог изделий. Источник для листа «Каталог» всех книг однолинейки</t>
   </si>
@@ -898,6 +898,24 @@
   </si>
   <si>
     <t>Контактор NXC-100 100А (AC-3) катушка AC230В</t>
+  </si>
+  <si>
+    <t>КМ NXC-120</t>
+  </si>
+  <si>
+    <t>Контактор NXC-120 120А (AC-3) катушка AC/DC230В</t>
+  </si>
+  <si>
+    <t>КМ NXC-160</t>
+  </si>
+  <si>
+    <t>Контактор NXC-160 160А (AC-3) катушка AC/DC230В</t>
+  </si>
+  <si>
+    <t>КМ NXC-185</t>
+  </si>
+  <si>
+    <t>Контактор NXC-185 185А (AC-3) катушка AC/DC230В</t>
   </si>
 </sst>
 </file>
@@ -1283,7 +1301,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q117"/>
+  <dimension ref="A1:Q120"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -3890,6 +3908,75 @@
         <v>24</v>
       </c>
     </row>
+    <row r="118" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>51</v>
+      </c>
+      <c r="B118" t="s">
+        <v>18</v>
+      </c>
+      <c r="C118" t="s">
+        <v>290</v>
+      </c>
+      <c r="G118" t="s">
+        <v>291</v>
+      </c>
+      <c r="I118" t="s">
+        <v>31</v>
+      </c>
+      <c r="J118">
+        <v>200</v>
+      </c>
+      <c r="M118" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="119" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>51</v>
+      </c>
+      <c r="B119" t="s">
+        <v>18</v>
+      </c>
+      <c r="C119" t="s">
+        <v>292</v>
+      </c>
+      <c r="G119" t="s">
+        <v>293</v>
+      </c>
+      <c r="I119" t="s">
+        <v>31</v>
+      </c>
+      <c r="J119">
+        <v>200</v>
+      </c>
+      <c r="M119" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="120" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>51</v>
+      </c>
+      <c r="B120" t="s">
+        <v>18</v>
+      </c>
+      <c r="C120" t="s">
+        <v>294</v>
+      </c>
+      <c r="G120" t="s">
+        <v>295</v>
+      </c>
+      <c r="I120" t="s">
+        <v>31</v>
+      </c>
+      <c r="J120">
+        <v>275</v>
+      </c>
+      <c r="M120" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:Q106" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>